<commit_message>
Add cards, columns, table blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (18):
- blocks/cards/cards.css
- blocks/columns/columns.css
- blocks/table/table.css
- scripts/scripts.js
- styles/lazy-styles.css
- templates/contactus/contactus.css
- templates/sidebar/sidebar.css
- tools/importer/PRODUCTS-QA-FINDINGS.md
- tools/importer/import-grace-master.bundle.js
- tools/importer/import-grace-master.js
- tools/importer/parsers/video-overlay.js
- tools/importer/reports/import-grace-master.report.xlsx
- tools/importer/reports/products/activcat-catalysts.report.json
- tools/importer/reports/products/consista.report.json
- tools/importer/reports/products/ludox.report.json
- tools/importer/reports/products/metallocenes.report.json
- tools/importer/reports/products/shieldex.report.json
- tools/importer/transformers/grace-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-grace-master.report.xlsx
+++ b/tools/importer/reports/import-grace-master.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3663" uniqueCount="1367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3664" uniqueCount="1366">
   <si>
     <t>_reportFile</t>
   </si>
@@ -2979,7 +2979,7 @@
     <t>products/activcat-catalysts</t>
   </si>
   <si>
-    <t>2026-08-09T21:25:15.988Z</t>
+    <t>2026-08-11T20:12:48.960Z</t>
   </si>
   <si>
     <t>ActivCat® Catalysts</t>
@@ -3024,7 +3024,7 @@
     <t>products/consista</t>
   </si>
   <si>
-    <t>2026-08-09T21:26:10.006Z</t>
+    <t>2026-08-11T20:07:35.632Z</t>
   </si>
   <si>
     <t>CONSISTA®</t>
@@ -3093,7 +3093,7 @@
     <t>products/ludox</t>
   </si>
   <si>
-    <t>2026-08-09T21:28:50.808Z</t>
+    <t>2026-08-11T16:54:11.193Z</t>
   </si>
   <si>
     <t>LUDOX®</t>
@@ -3153,10 +3153,7 @@
     <t>products/metallocenes</t>
   </si>
   <si>
-    <t>2026-08-09T21:32:23.242Z</t>
-  </si>
-  <si>
-    <t>Metallocenes</t>
+    <t>2026-08-11T20:16:13.549Z</t>
   </si>
   <si>
     <t>https://grace.com/products/metallocenes/</t>
@@ -3252,7 +3249,7 @@
     <t>products/shieldex</t>
   </si>
   <si>
-    <t>2026-08-09T21:36:39.463Z</t>
+    <t>2026-08-11T20:09:01.782Z</t>
   </si>
   <si>
     <t>SHIELDEX® Anti-Corrosive Pigments</t>
@@ -14522,10 +14519,10 @@
         <v>1044</v>
       </c>
       <c r="B201" t="s">
-        <v>979</v>
+        <v>19</v>
       </c>
       <c r="C201" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D201" t="s">
         <v>19</v>
@@ -14534,19 +14531,19 @@
         <v>19</v>
       </c>
       <c r="F201" t="s">
-        <v>19</v>
+        <v>323</v>
       </c>
       <c r="G201" t="s">
-        <v>19</v>
-      </c>
-      <c r="H201" t="b">
-        <v>0</v>
+        <v>324</v>
+      </c>
+      <c r="H201" t="s">
+        <v>19</v>
       </c>
       <c r="I201" t="s">
-        <v>980</v>
+        <v>19</v>
       </c>
       <c r="J201" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K201" t="s">
         <v>1045</v>
@@ -14555,21 +14552,21 @@
         <v>19</v>
       </c>
       <c r="M201" t="s">
-        <v>22</v>
+        <v>326</v>
       </c>
       <c r="N201" t="s">
         <v>1046</v>
       </c>
       <c r="O201" t="s">
+        <v>19</v>
+      </c>
+      <c r="P201" t="s">
         <v>1047</v>
-      </c>
-      <c r="P201" t="s">
-        <v>1048</v>
       </c>
     </row>
     <row r="202" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B202" t="s">
         <v>979</v>
@@ -14599,30 +14596,30 @@
         <v>20</v>
       </c>
       <c r="K202" t="s">
+        <v>1049</v>
+      </c>
+      <c r="L202" t="s">
+        <v>19</v>
+      </c>
+      <c r="M202" t="s">
+        <v>22</v>
+      </c>
+      <c r="N202" t="s">
         <v>1050</v>
       </c>
-      <c r="L202" t="s">
-        <v>19</v>
-      </c>
-      <c r="M202" t="s">
-        <v>22</v>
-      </c>
-      <c r="N202" t="s">
+      <c r="O202" t="s">
         <v>1051</v>
       </c>
-      <c r="O202" t="s">
+      <c r="P202" t="s">
         <v>1052</v>
-      </c>
-      <c r="P202" t="s">
-        <v>1053</v>
       </c>
     </row>
     <row r="203" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B203" t="s">
         <v>1054</v>
-      </c>
-      <c r="B203" t="s">
-        <v>1055</v>
       </c>
       <c r="C203" t="s">
         <v>18</v>
@@ -14649,7 +14646,7 @@
         <v>42</v>
       </c>
       <c r="K203" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="L203" t="b">
         <v>1</v>
@@ -14658,18 +14655,18 @@
         <v>22</v>
       </c>
       <c r="N203" t="s">
+        <v>1056</v>
+      </c>
+      <c r="O203" t="s">
         <v>1057</v>
       </c>
-      <c r="O203" t="s">
+      <c r="P203" t="s">
         <v>1058</v>
-      </c>
-      <c r="P203" t="s">
-        <v>1059</v>
       </c>
     </row>
     <row r="204" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B204" t="s">
         <v>18</v>
@@ -14699,7 +14696,7 @@
         <v>42</v>
       </c>
       <c r="K204" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="L204" t="b">
         <v>1</v>
@@ -14708,21 +14705,21 @@
         <v>22</v>
       </c>
       <c r="N204" t="s">
+        <v>1061</v>
+      </c>
+      <c r="O204" t="s">
         <v>1062</v>
       </c>
-      <c r="O204" t="s">
+      <c r="P204" t="s">
         <v>1063</v>
-      </c>
-      <c r="P204" t="s">
-        <v>1064</v>
       </c>
     </row>
     <row r="205" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B205" t="s">
         <v>1065</v>
-      </c>
-      <c r="B205" t="s">
-        <v>1066</v>
       </c>
       <c r="C205" t="s">
         <v>18</v>
@@ -14749,27 +14746,27 @@
         <v>20</v>
       </c>
       <c r="K205" t="s">
+        <v>1066</v>
+      </c>
+      <c r="L205" t="s">
+        <v>19</v>
+      </c>
+      <c r="M205" t="s">
+        <v>22</v>
+      </c>
+      <c r="N205" t="s">
         <v>1067</v>
       </c>
-      <c r="L205" t="s">
-        <v>19</v>
-      </c>
-      <c r="M205" t="s">
-        <v>22</v>
-      </c>
-      <c r="N205" t="s">
+      <c r="O205" t="s">
         <v>1068</v>
       </c>
-      <c r="O205" t="s">
+      <c r="P205" t="s">
         <v>1069</v>
-      </c>
-      <c r="P205" t="s">
-        <v>1070</v>
       </c>
     </row>
     <row r="206" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="B206" t="s">
         <v>979</v>
@@ -14799,30 +14796,30 @@
         <v>20</v>
       </c>
       <c r="K206" t="s">
+        <v>1071</v>
+      </c>
+      <c r="L206" t="s">
+        <v>19</v>
+      </c>
+      <c r="M206" t="s">
+        <v>22</v>
+      </c>
+      <c r="N206" t="s">
         <v>1072</v>
       </c>
-      <c r="L206" t="s">
-        <v>19</v>
-      </c>
-      <c r="M206" t="s">
-        <v>22</v>
-      </c>
-      <c r="N206" t="s">
+      <c r="O206" t="s">
         <v>1073</v>
       </c>
-      <c r="O206" t="s">
+      <c r="P206" t="s">
         <v>1074</v>
-      </c>
-      <c r="P206" t="s">
-        <v>1075</v>
       </c>
     </row>
     <row r="207" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
+        <v>1075</v>
+      </c>
+      <c r="B207" t="s">
         <v>1076</v>
-      </c>
-      <c r="B207" t="s">
-        <v>1077</v>
       </c>
       <c r="C207" t="s">
         <v>18</v>
@@ -14849,27 +14846,27 @@
         <v>20</v>
       </c>
       <c r="K207" t="s">
+        <v>1077</v>
+      </c>
+      <c r="L207" t="s">
+        <v>19</v>
+      </c>
+      <c r="M207" t="s">
+        <v>22</v>
+      </c>
+      <c r="N207" t="s">
         <v>1078</v>
       </c>
-      <c r="L207" t="s">
-        <v>19</v>
-      </c>
-      <c r="M207" t="s">
-        <v>22</v>
-      </c>
-      <c r="N207" t="s">
+      <c r="O207" t="s">
         <v>1079</v>
       </c>
-      <c r="O207" t="s">
+      <c r="P207" t="s">
         <v>1080</v>
-      </c>
-      <c r="P207" t="s">
-        <v>1081</v>
       </c>
     </row>
     <row r="208" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="B208" t="s">
         <v>1024</v>
@@ -14899,30 +14896,30 @@
         <v>20</v>
       </c>
       <c r="K208" t="s">
+        <v>1082</v>
+      </c>
+      <c r="L208" t="s">
+        <v>19</v>
+      </c>
+      <c r="M208" t="s">
+        <v>22</v>
+      </c>
+      <c r="N208" t="s">
         <v>1083</v>
       </c>
-      <c r="L208" t="s">
-        <v>19</v>
-      </c>
-      <c r="M208" t="s">
-        <v>22</v>
-      </c>
-      <c r="N208" t="s">
+      <c r="O208" t="s">
         <v>1084</v>
       </c>
-      <c r="O208" t="s">
+      <c r="P208" t="s">
         <v>1085</v>
-      </c>
-      <c r="P208" t="s">
-        <v>1086</v>
       </c>
     </row>
     <row r="209" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="B209" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C209" t="s">
         <v>18</v>
@@ -14949,30 +14946,30 @@
         <v>20</v>
       </c>
       <c r="K209" t="s">
+        <v>1087</v>
+      </c>
+      <c r="L209" t="s">
+        <v>19</v>
+      </c>
+      <c r="M209" t="s">
+        <v>22</v>
+      </c>
+      <c r="N209" t="s">
         <v>1088</v>
       </c>
-      <c r="L209" t="s">
-        <v>19</v>
-      </c>
-      <c r="M209" t="s">
-        <v>22</v>
-      </c>
-      <c r="N209" t="s">
+      <c r="O209" t="s">
         <v>1089</v>
       </c>
-      <c r="O209" t="s">
+      <c r="P209" t="s">
         <v>1090</v>
-      </c>
-      <c r="P209" t="s">
-        <v>1091</v>
       </c>
     </row>
     <row r="210" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="B210" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C210" t="s">
         <v>18</v>
@@ -14999,30 +14996,30 @@
         <v>20</v>
       </c>
       <c r="K210" t="s">
+        <v>1092</v>
+      </c>
+      <c r="L210" t="s">
+        <v>19</v>
+      </c>
+      <c r="M210" t="s">
+        <v>22</v>
+      </c>
+      <c r="N210" t="s">
         <v>1093</v>
       </c>
-      <c r="L210" t="s">
-        <v>19</v>
-      </c>
-      <c r="M210" t="s">
-        <v>22</v>
-      </c>
-      <c r="N210" t="s">
+      <c r="O210" t="s">
         <v>1094</v>
       </c>
-      <c r="O210" t="s">
+      <c r="P210" t="s">
         <v>1095</v>
-      </c>
-      <c r="P210" t="s">
-        <v>1096</v>
       </c>
     </row>
     <row r="211" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B211" t="s">
         <v>1097</v>
-      </c>
-      <c r="B211" t="s">
-        <v>1098</v>
       </c>
       <c r="C211" t="s">
         <v>18</v>
@@ -15049,30 +15046,30 @@
         <v>20</v>
       </c>
       <c r="K211" t="s">
+        <v>1098</v>
+      </c>
+      <c r="L211" t="s">
+        <v>19</v>
+      </c>
+      <c r="M211" t="s">
+        <v>22</v>
+      </c>
+      <c r="N211" t="s">
         <v>1099</v>
       </c>
-      <c r="L211" t="s">
-        <v>19</v>
-      </c>
-      <c r="M211" t="s">
-        <v>22</v>
-      </c>
-      <c r="N211" t="s">
+      <c r="O211" t="s">
         <v>1100</v>
       </c>
-      <c r="O211" t="s">
+      <c r="P211" t="s">
         <v>1101</v>
-      </c>
-      <c r="P211" t="s">
-        <v>1102</v>
       </c>
     </row>
     <row r="212" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="B212" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C212" t="s">
         <v>18</v>
@@ -15099,27 +15096,27 @@
         <v>20</v>
       </c>
       <c r="K212" t="s">
+        <v>1103</v>
+      </c>
+      <c r="L212" t="s">
+        <v>19</v>
+      </c>
+      <c r="M212" t="s">
+        <v>22</v>
+      </c>
+      <c r="N212" t="s">
         <v>1104</v>
       </c>
-      <c r="L212" t="s">
-        <v>19</v>
-      </c>
-      <c r="M212" t="s">
-        <v>22</v>
-      </c>
-      <c r="N212" t="s">
+      <c r="O212" t="s">
         <v>1105</v>
       </c>
-      <c r="O212" t="s">
+      <c r="P212" t="s">
         <v>1106</v>
-      </c>
-      <c r="P212" t="s">
-        <v>1107</v>
       </c>
     </row>
     <row r="213" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="B213" t="s">
         <v>979</v>
@@ -15149,27 +15146,27 @@
         <v>20</v>
       </c>
       <c r="K213" t="s">
+        <v>1108</v>
+      </c>
+      <c r="L213" t="s">
+        <v>19</v>
+      </c>
+      <c r="M213" t="s">
+        <v>22</v>
+      </c>
+      <c r="N213" t="s">
         <v>1109</v>
       </c>
-      <c r="L213" t="s">
-        <v>19</v>
-      </c>
-      <c r="M213" t="s">
-        <v>22</v>
-      </c>
-      <c r="N213" t="s">
+      <c r="O213" t="s">
         <v>1110</v>
       </c>
-      <c r="O213" t="s">
+      <c r="P213" t="s">
         <v>1111</v>
-      </c>
-      <c r="P213" t="s">
-        <v>1112</v>
       </c>
     </row>
     <row r="214" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B214" t="s">
         <v>979</v>
@@ -15199,27 +15196,27 @@
         <v>20</v>
       </c>
       <c r="K214" t="s">
+        <v>1113</v>
+      </c>
+      <c r="L214" t="s">
+        <v>19</v>
+      </c>
+      <c r="M214" t="s">
+        <v>22</v>
+      </c>
+      <c r="N214" t="s">
         <v>1114</v>
       </c>
-      <c r="L214" t="s">
-        <v>19</v>
-      </c>
-      <c r="M214" t="s">
-        <v>22</v>
-      </c>
-      <c r="N214" t="s">
+      <c r="O214" t="s">
         <v>1115</v>
       </c>
-      <c r="O214" t="s">
+      <c r="P214" t="s">
         <v>1116</v>
-      </c>
-      <c r="P214" t="s">
-        <v>1117</v>
       </c>
     </row>
     <row r="215" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="B215" t="s">
         <v>1024</v>
@@ -15249,27 +15246,27 @@
         <v>20</v>
       </c>
       <c r="K215" t="s">
+        <v>1118</v>
+      </c>
+      <c r="L215" t="s">
+        <v>19</v>
+      </c>
+      <c r="M215" t="s">
+        <v>22</v>
+      </c>
+      <c r="N215" t="s">
         <v>1119</v>
       </c>
-      <c r="L215" t="s">
-        <v>19</v>
-      </c>
-      <c r="M215" t="s">
-        <v>22</v>
-      </c>
-      <c r="N215" t="s">
+      <c r="O215" t="s">
         <v>1120</v>
       </c>
-      <c r="O215" t="s">
+      <c r="P215" t="s">
         <v>1121</v>
-      </c>
-      <c r="P215" t="s">
-        <v>1122</v>
       </c>
     </row>
     <row r="216" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="B216" t="s">
         <v>18</v>
@@ -15299,7 +15296,7 @@
         <v>42</v>
       </c>
       <c r="K216" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="L216" t="b">
         <v>1</v>
@@ -15308,21 +15305,21 @@
         <v>22</v>
       </c>
       <c r="N216" t="s">
+        <v>1124</v>
+      </c>
+      <c r="O216" t="s">
         <v>1125</v>
       </c>
-      <c r="O216" t="s">
+      <c r="P216" t="s">
         <v>1126</v>
-      </c>
-      <c r="P216" t="s">
-        <v>1127</v>
       </c>
     </row>
     <row r="217" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B217" t="s">
         <v>1128</v>
-      </c>
-      <c r="B217" t="s">
-        <v>1129</v>
       </c>
       <c r="C217" t="s">
         <v>18</v>
@@ -15349,30 +15346,30 @@
         <v>20</v>
       </c>
       <c r="K217" t="s">
+        <v>1129</v>
+      </c>
+      <c r="L217" t="s">
+        <v>19</v>
+      </c>
+      <c r="M217" t="s">
+        <v>22</v>
+      </c>
+      <c r="N217" t="s">
         <v>1130</v>
       </c>
-      <c r="L217" t="s">
-        <v>19</v>
-      </c>
-      <c r="M217" t="s">
-        <v>22</v>
-      </c>
-      <c r="N217" t="s">
+      <c r="O217" t="s">
         <v>1131</v>
       </c>
-      <c r="O217" t="s">
+      <c r="P217" t="s">
         <v>1132</v>
-      </c>
-      <c r="P217" t="s">
-        <v>1133</v>
       </c>
     </row>
     <row r="218" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B218" t="s">
         <v>1134</v>
-      </c>
-      <c r="B218" t="s">
-        <v>1135</v>
       </c>
       <c r="C218" t="s">
         <v>18</v>
@@ -15399,27 +15396,27 @@
         <v>20</v>
       </c>
       <c r="K218" t="s">
+        <v>1135</v>
+      </c>
+      <c r="L218" t="s">
+        <v>19</v>
+      </c>
+      <c r="M218" t="s">
+        <v>22</v>
+      </c>
+      <c r="N218" t="s">
         <v>1136</v>
       </c>
-      <c r="L218" t="s">
-        <v>19</v>
-      </c>
-      <c r="M218" t="s">
-        <v>22</v>
-      </c>
-      <c r="N218" t="s">
+      <c r="O218" t="s">
         <v>1137</v>
       </c>
-      <c r="O218" t="s">
+      <c r="P218" t="s">
         <v>1138</v>
-      </c>
-      <c r="P218" t="s">
-        <v>1139</v>
       </c>
     </row>
     <row r="219" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="B219" t="s">
         <v>979</v>
@@ -15449,30 +15446,30 @@
         <v>20</v>
       </c>
       <c r="K219" t="s">
+        <v>1140</v>
+      </c>
+      <c r="L219" t="s">
+        <v>19</v>
+      </c>
+      <c r="M219" t="s">
+        <v>22</v>
+      </c>
+      <c r="N219" t="s">
         <v>1141</v>
       </c>
-      <c r="L219" t="s">
-        <v>19</v>
-      </c>
-      <c r="M219" t="s">
-        <v>22</v>
-      </c>
-      <c r="N219" t="s">
+      <c r="O219" t="s">
         <v>1142</v>
       </c>
-      <c r="O219" t="s">
+      <c r="P219" t="s">
         <v>1143</v>
-      </c>
-      <c r="P219" t="s">
-        <v>1144</v>
       </c>
     </row>
     <row r="220" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
+        <v>1144</v>
+      </c>
+      <c r="B220" t="s">
         <v>1145</v>
-      </c>
-      <c r="B220" t="s">
-        <v>1146</v>
       </c>
       <c r="C220" t="s">
         <v>18</v>
@@ -15499,27 +15496,27 @@
         <v>20</v>
       </c>
       <c r="K220" t="s">
+        <v>1146</v>
+      </c>
+      <c r="L220" t="s">
+        <v>19</v>
+      </c>
+      <c r="M220" t="s">
+        <v>22</v>
+      </c>
+      <c r="N220" t="s">
         <v>1147</v>
       </c>
-      <c r="L220" t="s">
-        <v>19</v>
-      </c>
-      <c r="M220" t="s">
-        <v>22</v>
-      </c>
-      <c r="N220" t="s">
+      <c r="O220" t="s">
         <v>1148</v>
       </c>
-      <c r="O220" t="s">
+      <c r="P220" t="s">
         <v>1149</v>
-      </c>
-      <c r="P220" t="s">
-        <v>1150</v>
       </c>
     </row>
     <row r="221" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="B221" t="s">
         <v>979</v>
@@ -15549,30 +15546,30 @@
         <v>20</v>
       </c>
       <c r="K221" t="s">
+        <v>1151</v>
+      </c>
+      <c r="L221" t="s">
+        <v>19</v>
+      </c>
+      <c r="M221" t="s">
+        <v>22</v>
+      </c>
+      <c r="N221" t="s">
         <v>1152</v>
       </c>
-      <c r="L221" t="s">
-        <v>19</v>
-      </c>
-      <c r="M221" t="s">
-        <v>22</v>
-      </c>
-      <c r="N221" t="s">
+      <c r="O221" t="s">
         <v>1153</v>
       </c>
-      <c r="O221" t="s">
+      <c r="P221" t="s">
         <v>1154</v>
-      </c>
-      <c r="P221" t="s">
-        <v>1155</v>
       </c>
     </row>
     <row r="222" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
+        <v>1155</v>
+      </c>
+      <c r="B222" t="s">
         <v>1156</v>
-      </c>
-      <c r="B222" t="s">
-        <v>1157</v>
       </c>
       <c r="C222" t="s">
         <v>18</v>
@@ -15599,33 +15596,33 @@
         <v>20</v>
       </c>
       <c r="K222" t="s">
+        <v>1157</v>
+      </c>
+      <c r="L222" t="s">
+        <v>19</v>
+      </c>
+      <c r="M222" t="s">
+        <v>22</v>
+      </c>
+      <c r="N222" t="s">
         <v>1158</v>
       </c>
-      <c r="L222" t="s">
-        <v>19</v>
-      </c>
-      <c r="M222" t="s">
-        <v>22</v>
-      </c>
-      <c r="N222" t="s">
+      <c r="O222" t="s">
         <v>1159</v>
       </c>
-      <c r="O222" t="s">
+      <c r="P222" t="s">
         <v>1160</v>
-      </c>
-      <c r="P222" t="s">
-        <v>1161</v>
       </c>
     </row>
     <row r="223" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B223" t="s">
         <v>1162</v>
       </c>
-      <c r="B223" t="s">
+      <c r="C223" t="s">
         <v>1163</v>
-      </c>
-      <c r="C223" t="s">
-        <v>1164</v>
       </c>
       <c r="D223" t="s">
         <v>19</v>
@@ -15649,30 +15646,30 @@
         <v>20</v>
       </c>
       <c r="K223" t="s">
+        <v>1164</v>
+      </c>
+      <c r="L223" t="s">
+        <v>19</v>
+      </c>
+      <c r="M223" t="s">
+        <v>22</v>
+      </c>
+      <c r="N223" t="s">
         <v>1165</v>
       </c>
-      <c r="L223" t="s">
-        <v>19</v>
-      </c>
-      <c r="M223" t="s">
-        <v>22</v>
-      </c>
-      <c r="N223" t="s">
+      <c r="O223" t="s">
         <v>1166</v>
       </c>
-      <c r="O223" t="s">
+      <c r="P223" t="s">
         <v>1167</v>
-      </c>
-      <c r="P223" t="s">
-        <v>1168</v>
       </c>
     </row>
     <row r="224" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B224" t="s">
         <v>1169</v>
-      </c>
-      <c r="B224" t="s">
-        <v>1170</v>
       </c>
       <c r="C224" t="s">
         <v>18</v>
@@ -15699,7 +15696,7 @@
         <v>42</v>
       </c>
       <c r="K224" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="L224" t="b">
         <v>0</v>
@@ -15708,21 +15705,21 @@
         <v>22</v>
       </c>
       <c r="N224" t="s">
+        <v>1171</v>
+      </c>
+      <c r="O224" t="s">
         <v>1172</v>
       </c>
-      <c r="O224" t="s">
+      <c r="P224" t="s">
         <v>1173</v>
-      </c>
-      <c r="P224" t="s">
-        <v>1174</v>
       </c>
     </row>
     <row r="225" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B225" t="s">
         <v>1175</v>
-      </c>
-      <c r="B225" t="s">
-        <v>1176</v>
       </c>
       <c r="C225" t="s">
         <v>129</v>
@@ -15749,7 +15746,7 @@
         <v>42</v>
       </c>
       <c r="K225" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="L225" t="b">
         <v>1</v>
@@ -15758,21 +15755,21 @@
         <v>22</v>
       </c>
       <c r="N225" t="s">
+        <v>1177</v>
+      </c>
+      <c r="O225" t="s">
         <v>1178</v>
       </c>
-      <c r="O225" t="s">
+      <c r="P225" t="s">
         <v>1179</v>
-      </c>
-      <c r="P225" t="s">
-        <v>1180</v>
       </c>
     </row>
     <row r="226" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
+        <v>1180</v>
+      </c>
+      <c r="B226" t="s">
         <v>1181</v>
-      </c>
-      <c r="B226" t="s">
-        <v>1182</v>
       </c>
       <c r="C226" t="s">
         <v>18</v>
@@ -15799,7 +15796,7 @@
         <v>42</v>
       </c>
       <c r="K226" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="L226" t="b">
         <v>1</v>
@@ -15808,21 +15805,21 @@
         <v>22</v>
       </c>
       <c r="N226" t="s">
+        <v>1183</v>
+      </c>
+      <c r="O226" t="s">
         <v>1184</v>
       </c>
-      <c r="O226" t="s">
+      <c r="P226" t="s">
         <v>1185</v>
-      </c>
-      <c r="P226" t="s">
-        <v>1186</v>
       </c>
     </row>
     <row r="227" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
+        <v>1186</v>
+      </c>
+      <c r="B227" t="s">
         <v>1187</v>
-      </c>
-      <c r="B227" t="s">
-        <v>1188</v>
       </c>
       <c r="C227" t="s">
         <v>18</v>
@@ -15849,30 +15846,30 @@
         <v>20</v>
       </c>
       <c r="K227" t="s">
+        <v>1188</v>
+      </c>
+      <c r="L227" t="s">
+        <v>19</v>
+      </c>
+      <c r="M227" t="s">
+        <v>22</v>
+      </c>
+      <c r="N227" t="s">
         <v>1189</v>
       </c>
-      <c r="L227" t="s">
-        <v>19</v>
-      </c>
-      <c r="M227" t="s">
-        <v>22</v>
-      </c>
-      <c r="N227" t="s">
+      <c r="O227" t="s">
         <v>1190</v>
       </c>
-      <c r="O227" t="s">
+      <c r="P227" t="s">
         <v>1191</v>
-      </c>
-      <c r="P227" t="s">
-        <v>1192</v>
       </c>
     </row>
     <row r="228" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
+        <v>1192</v>
+      </c>
+      <c r="B228" t="s">
         <v>1193</v>
-      </c>
-      <c r="B228" t="s">
-        <v>1194</v>
       </c>
       <c r="C228" t="s">
         <v>18</v>
@@ -15899,30 +15896,30 @@
         <v>20</v>
       </c>
       <c r="K228" t="s">
+        <v>1194</v>
+      </c>
+      <c r="L228" t="s">
+        <v>19</v>
+      </c>
+      <c r="M228" t="s">
+        <v>22</v>
+      </c>
+      <c r="N228" t="s">
         <v>1195</v>
       </c>
-      <c r="L228" t="s">
-        <v>19</v>
-      </c>
-      <c r="M228" t="s">
-        <v>22</v>
-      </c>
-      <c r="N228" t="s">
+      <c r="O228" t="s">
         <v>1196</v>
       </c>
-      <c r="O228" t="s">
+      <c r="P228" t="s">
         <v>1197</v>
-      </c>
-      <c r="P228" t="s">
-        <v>1198</v>
       </c>
     </row>
     <row r="229" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B229" t="s">
         <v>1199</v>
-      </c>
-      <c r="B229" t="s">
-        <v>1200</v>
       </c>
       <c r="C229" t="s">
         <v>40</v>
@@ -15949,7 +15946,7 @@
         <v>42</v>
       </c>
       <c r="K229" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="L229" t="b">
         <v>1</v>
@@ -15958,21 +15955,21 @@
         <v>22</v>
       </c>
       <c r="N229" t="s">
+        <v>1201</v>
+      </c>
+      <c r="O229" t="s">
         <v>1202</v>
       </c>
-      <c r="O229" t="s">
+      <c r="P229" t="s">
         <v>1203</v>
-      </c>
-      <c r="P229" t="s">
-        <v>1204</v>
       </c>
     </row>
     <row r="230" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
+        <v>1204</v>
+      </c>
+      <c r="B230" t="s">
         <v>1205</v>
-      </c>
-      <c r="B230" t="s">
-        <v>1206</v>
       </c>
       <c r="C230" t="s">
         <v>18</v>
@@ -15993,39 +15990,39 @@
         <v>0</v>
       </c>
       <c r="I230" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J230" t="s">
         <v>20</v>
       </c>
       <c r="K230" t="s">
+        <v>1207</v>
+      </c>
+      <c r="L230" t="s">
+        <v>19</v>
+      </c>
+      <c r="M230" t="s">
+        <v>22</v>
+      </c>
+      <c r="N230" t="s">
         <v>1208</v>
       </c>
-      <c r="L230" t="s">
-        <v>19</v>
-      </c>
-      <c r="M230" t="s">
-        <v>22</v>
-      </c>
-      <c r="N230" t="s">
+      <c r="O230" t="s">
         <v>1209</v>
       </c>
-      <c r="O230" t="s">
+      <c r="P230" t="s">
         <v>1210</v>
-      </c>
-      <c r="P230" t="s">
-        <v>1211</v>
       </c>
     </row>
     <row r="231" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
+        <v>1211</v>
+      </c>
+      <c r="B231" t="s">
         <v>1212</v>
       </c>
-      <c r="B231" t="s">
+      <c r="C231" t="s">
         <v>1213</v>
-      </c>
-      <c r="C231" t="s">
-        <v>1214</v>
       </c>
       <c r="D231" t="b">
         <v>0</v>
@@ -16049,7 +16046,7 @@
         <v>42</v>
       </c>
       <c r="K231" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="L231" t="b">
         <v>1</v>
@@ -16058,24 +16055,24 @@
         <v>22</v>
       </c>
       <c r="N231" t="s">
+        <v>1215</v>
+      </c>
+      <c r="O231" t="s">
         <v>1216</v>
       </c>
-      <c r="O231" t="s">
+      <c r="P231" t="s">
         <v>1217</v>
-      </c>
-      <c r="P231" t="s">
-        <v>1218</v>
       </c>
     </row>
     <row r="232" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
+        <v>1218</v>
+      </c>
+      <c r="B232" t="s">
         <v>1219</v>
       </c>
-      <c r="B232" t="s">
+      <c r="C232" t="s">
         <v>1220</v>
-      </c>
-      <c r="C232" t="s">
-        <v>1221</v>
       </c>
       <c r="D232" t="b">
         <v>0</v>
@@ -16099,7 +16096,7 @@
         <v>42</v>
       </c>
       <c r="K232" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="L232" t="b">
         <v>1</v>
@@ -16108,21 +16105,21 @@
         <v>22</v>
       </c>
       <c r="N232" t="s">
+        <v>1222</v>
+      </c>
+      <c r="O232" t="s">
         <v>1223</v>
       </c>
-      <c r="O232" t="s">
+      <c r="P232" t="s">
         <v>1224</v>
-      </c>
-      <c r="P232" t="s">
-        <v>1225</v>
       </c>
     </row>
     <row r="233" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
+        <v>1225</v>
+      </c>
+      <c r="B233" t="s">
         <v>1226</v>
-      </c>
-      <c r="B233" t="s">
-        <v>1227</v>
       </c>
       <c r="C233" t="s">
         <v>18</v>
@@ -16149,30 +16146,30 @@
         <v>20</v>
       </c>
       <c r="K233" t="s">
+        <v>1227</v>
+      </c>
+      <c r="L233" t="s">
+        <v>19</v>
+      </c>
+      <c r="M233" t="s">
+        <v>22</v>
+      </c>
+      <c r="N233" t="s">
         <v>1228</v>
       </c>
-      <c r="L233" t="s">
-        <v>19</v>
-      </c>
-      <c r="M233" t="s">
-        <v>22</v>
-      </c>
-      <c r="N233" t="s">
+      <c r="O233" t="s">
         <v>1229</v>
       </c>
-      <c r="O233" t="s">
+      <c r="P233" t="s">
         <v>1230</v>
-      </c>
-      <c r="P233" t="s">
-        <v>1231</v>
       </c>
     </row>
     <row r="234" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="B234" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C234" t="s">
         <v>18</v>
@@ -16199,30 +16196,30 @@
         <v>20</v>
       </c>
       <c r="K234" t="s">
+        <v>1232</v>
+      </c>
+      <c r="L234" t="s">
+        <v>19</v>
+      </c>
+      <c r="M234" t="s">
+        <v>22</v>
+      </c>
+      <c r="N234" t="s">
         <v>1233</v>
       </c>
-      <c r="L234" t="s">
-        <v>19</v>
-      </c>
-      <c r="M234" t="s">
-        <v>22</v>
-      </c>
-      <c r="N234" t="s">
+      <c r="O234" t="s">
         <v>1234</v>
       </c>
-      <c r="O234" t="s">
+      <c r="P234" t="s">
         <v>1235</v>
-      </c>
-      <c r="P234" t="s">
-        <v>1236</v>
       </c>
     </row>
     <row r="235" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="B235" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C235" t="s">
         <v>18</v>
@@ -16249,30 +16246,30 @@
         <v>20</v>
       </c>
       <c r="K235" t="s">
+        <v>1237</v>
+      </c>
+      <c r="L235" t="s">
+        <v>19</v>
+      </c>
+      <c r="M235" t="s">
+        <v>22</v>
+      </c>
+      <c r="N235" t="s">
         <v>1238</v>
       </c>
-      <c r="L235" t="s">
-        <v>19</v>
-      </c>
-      <c r="M235" t="s">
-        <v>22</v>
-      </c>
-      <c r="N235" t="s">
+      <c r="O235" t="s">
         <v>1239</v>
       </c>
-      <c r="O235" t="s">
+      <c r="P235" t="s">
         <v>1240</v>
-      </c>
-      <c r="P235" t="s">
-        <v>1241</v>
       </c>
     </row>
     <row r="236" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="B236" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C236" t="s">
         <v>18</v>
@@ -16299,30 +16296,30 @@
         <v>20</v>
       </c>
       <c r="K236" t="s">
+        <v>1242</v>
+      </c>
+      <c r="L236" t="s">
+        <v>19</v>
+      </c>
+      <c r="M236" t="s">
+        <v>22</v>
+      </c>
+      <c r="N236" t="s">
         <v>1243</v>
       </c>
-      <c r="L236" t="s">
-        <v>19</v>
-      </c>
-      <c r="M236" t="s">
-        <v>22</v>
-      </c>
-      <c r="N236" t="s">
+      <c r="O236" t="s">
         <v>1244</v>
       </c>
-      <c r="O236" t="s">
+      <c r="P236" t="s">
         <v>1245</v>
-      </c>
-      <c r="P236" t="s">
-        <v>1246</v>
       </c>
     </row>
     <row r="237" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="B237" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C237" t="s">
         <v>18</v>
@@ -16349,30 +16346,30 @@
         <v>20</v>
       </c>
       <c r="K237" t="s">
+        <v>1247</v>
+      </c>
+      <c r="L237" t="s">
+        <v>19</v>
+      </c>
+      <c r="M237" t="s">
+        <v>22</v>
+      </c>
+      <c r="N237" t="s">
         <v>1248</v>
       </c>
-      <c r="L237" t="s">
-        <v>19</v>
-      </c>
-      <c r="M237" t="s">
-        <v>22</v>
-      </c>
-      <c r="N237" t="s">
+      <c r="O237" t="s">
         <v>1249</v>
       </c>
-      <c r="O237" t="s">
+      <c r="P237" t="s">
         <v>1250</v>
-      </c>
-      <c r="P237" t="s">
-        <v>1251</v>
       </c>
     </row>
     <row r="238" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="B238" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C238" t="s">
         <v>18</v>
@@ -16399,30 +16396,30 @@
         <v>20</v>
       </c>
       <c r="K238" t="s">
+        <v>1252</v>
+      </c>
+      <c r="L238" t="s">
+        <v>19</v>
+      </c>
+      <c r="M238" t="s">
+        <v>22</v>
+      </c>
+      <c r="N238" t="s">
         <v>1253</v>
       </c>
-      <c r="L238" t="s">
-        <v>19</v>
-      </c>
-      <c r="M238" t="s">
-        <v>22</v>
-      </c>
-      <c r="N238" t="s">
+      <c r="O238" t="s">
         <v>1254</v>
       </c>
-      <c r="O238" t="s">
+      <c r="P238" t="s">
         <v>1255</v>
-      </c>
-      <c r="P238" t="s">
-        <v>1256</v>
       </c>
     </row>
     <row r="239" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="B239" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C239" t="s">
         <v>18</v>
@@ -16449,30 +16446,30 @@
         <v>20</v>
       </c>
       <c r="K239" t="s">
+        <v>1257</v>
+      </c>
+      <c r="L239" t="s">
+        <v>19</v>
+      </c>
+      <c r="M239" t="s">
+        <v>22</v>
+      </c>
+      <c r="N239" t="s">
         <v>1258</v>
       </c>
-      <c r="L239" t="s">
-        <v>19</v>
-      </c>
-      <c r="M239" t="s">
-        <v>22</v>
-      </c>
-      <c r="N239" t="s">
+      <c r="O239" t="s">
         <v>1259</v>
       </c>
-      <c r="O239" t="s">
+      <c r="P239" t="s">
         <v>1260</v>
-      </c>
-      <c r="P239" t="s">
-        <v>1261</v>
       </c>
     </row>
     <row r="240" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="B240" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C240" t="s">
         <v>18</v>
@@ -16499,30 +16496,30 @@
         <v>20</v>
       </c>
       <c r="K240" t="s">
+        <v>1262</v>
+      </c>
+      <c r="L240" t="s">
+        <v>19</v>
+      </c>
+      <c r="M240" t="s">
+        <v>22</v>
+      </c>
+      <c r="N240" t="s">
         <v>1263</v>
       </c>
-      <c r="L240" t="s">
-        <v>19</v>
-      </c>
-      <c r="M240" t="s">
-        <v>22</v>
-      </c>
-      <c r="N240" t="s">
+      <c r="O240" t="s">
         <v>1264</v>
       </c>
-      <c r="O240" t="s">
+      <c r="P240" t="s">
         <v>1265</v>
-      </c>
-      <c r="P240" t="s">
-        <v>1266</v>
       </c>
     </row>
     <row r="241" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="B241" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C241" t="s">
         <v>18</v>
@@ -16549,30 +16546,30 @@
         <v>20</v>
       </c>
       <c r="K241" t="s">
+        <v>1267</v>
+      </c>
+      <c r="L241" t="s">
+        <v>19</v>
+      </c>
+      <c r="M241" t="s">
+        <v>22</v>
+      </c>
+      <c r="N241" t="s">
         <v>1268</v>
       </c>
-      <c r="L241" t="s">
-        <v>19</v>
-      </c>
-      <c r="M241" t="s">
-        <v>22</v>
-      </c>
-      <c r="N241" t="s">
+      <c r="O241" t="s">
         <v>1269</v>
       </c>
-      <c r="O241" t="s">
+      <c r="P241" t="s">
         <v>1270</v>
-      </c>
-      <c r="P241" t="s">
-        <v>1271</v>
       </c>
     </row>
     <row r="242" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
       <c r="B242" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C242" t="s">
         <v>18</v>
@@ -16599,30 +16596,30 @@
         <v>20</v>
       </c>
       <c r="K242" t="s">
+        <v>1272</v>
+      </c>
+      <c r="L242" t="s">
+        <v>19</v>
+      </c>
+      <c r="M242" t="s">
+        <v>22</v>
+      </c>
+      <c r="N242" t="s">
         <v>1273</v>
       </c>
-      <c r="L242" t="s">
-        <v>19</v>
-      </c>
-      <c r="M242" t="s">
-        <v>22</v>
-      </c>
-      <c r="N242" t="s">
+      <c r="O242" t="s">
         <v>1274</v>
       </c>
-      <c r="O242" t="s">
+      <c r="P242" t="s">
         <v>1275</v>
-      </c>
-      <c r="P242" t="s">
-        <v>1276</v>
       </c>
     </row>
     <row r="243" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="B243" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C243" t="s">
         <v>18</v>
@@ -16649,30 +16646,30 @@
         <v>20</v>
       </c>
       <c r="K243" t="s">
+        <v>1277</v>
+      </c>
+      <c r="L243" t="s">
+        <v>19</v>
+      </c>
+      <c r="M243" t="s">
+        <v>22</v>
+      </c>
+      <c r="N243" t="s">
         <v>1278</v>
       </c>
-      <c r="L243" t="s">
-        <v>19</v>
-      </c>
-      <c r="M243" t="s">
-        <v>22</v>
-      </c>
-      <c r="N243" t="s">
+      <c r="O243" t="s">
         <v>1279</v>
       </c>
-      <c r="O243" t="s">
+      <c r="P243" t="s">
         <v>1280</v>
-      </c>
-      <c r="P243" t="s">
-        <v>1281</v>
       </c>
     </row>
     <row r="244" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="B244" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C244" t="s">
         <v>18</v>
@@ -16699,30 +16696,30 @@
         <v>20</v>
       </c>
       <c r="K244" t="s">
+        <v>1282</v>
+      </c>
+      <c r="L244" t="s">
+        <v>19</v>
+      </c>
+      <c r="M244" t="s">
+        <v>22</v>
+      </c>
+      <c r="N244" t="s">
         <v>1283</v>
       </c>
-      <c r="L244" t="s">
-        <v>19</v>
-      </c>
-      <c r="M244" t="s">
-        <v>22</v>
-      </c>
-      <c r="N244" t="s">
+      <c r="O244" t="s">
         <v>1284</v>
       </c>
-      <c r="O244" t="s">
+      <c r="P244" t="s">
         <v>1285</v>
-      </c>
-      <c r="P244" t="s">
-        <v>1286</v>
       </c>
     </row>
     <row r="245" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="B245" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C245" t="s">
         <v>18</v>
@@ -16743,36 +16740,36 @@
         <v>0</v>
       </c>
       <c r="I245" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J245" t="s">
         <v>20</v>
       </c>
       <c r="K245" t="s">
+        <v>1287</v>
+      </c>
+      <c r="L245" t="s">
+        <v>19</v>
+      </c>
+      <c r="M245" t="s">
+        <v>22</v>
+      </c>
+      <c r="N245" t="s">
         <v>1288</v>
       </c>
-      <c r="L245" t="s">
-        <v>19</v>
-      </c>
-      <c r="M245" t="s">
-        <v>22</v>
-      </c>
-      <c r="N245" t="s">
+      <c r="O245" t="s">
         <v>1289</v>
       </c>
-      <c r="O245" t="s">
+      <c r="P245" t="s">
         <v>1290</v>
-      </c>
-      <c r="P245" t="s">
-        <v>1291</v>
       </c>
     </row>
     <row r="246" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="B246" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C246" t="s">
         <v>18</v>
@@ -16793,36 +16790,36 @@
         <v>0</v>
       </c>
       <c r="I246" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J246" t="s">
         <v>20</v>
       </c>
       <c r="K246" t="s">
+        <v>1292</v>
+      </c>
+      <c r="L246" t="s">
+        <v>19</v>
+      </c>
+      <c r="M246" t="s">
+        <v>22</v>
+      </c>
+      <c r="N246" t="s">
         <v>1293</v>
       </c>
-      <c r="L246" t="s">
-        <v>19</v>
-      </c>
-      <c r="M246" t="s">
-        <v>22</v>
-      </c>
-      <c r="N246" t="s">
+      <c r="O246" t="s">
         <v>1294</v>
       </c>
-      <c r="O246" t="s">
+      <c r="P246" t="s">
         <v>1295</v>
-      </c>
-      <c r="P246" t="s">
-        <v>1296</v>
       </c>
     </row>
     <row r="247" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="B247" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C247" t="s">
         <v>18</v>
@@ -16843,36 +16840,36 @@
         <v>0</v>
       </c>
       <c r="I247" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J247" t="s">
         <v>20</v>
       </c>
       <c r="K247" t="s">
+        <v>1297</v>
+      </c>
+      <c r="L247" t="s">
+        <v>19</v>
+      </c>
+      <c r="M247" t="s">
+        <v>22</v>
+      </c>
+      <c r="N247" t="s">
         <v>1298</v>
       </c>
-      <c r="L247" t="s">
-        <v>19</v>
-      </c>
-      <c r="M247" t="s">
-        <v>22</v>
-      </c>
-      <c r="N247" t="s">
+      <c r="O247" t="s">
         <v>1299</v>
       </c>
-      <c r="O247" t="s">
+      <c r="P247" t="s">
         <v>1300</v>
-      </c>
-      <c r="P247" t="s">
-        <v>1301</v>
       </c>
     </row>
     <row r="248" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="B248" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C248" t="s">
         <v>18</v>
@@ -16893,36 +16890,36 @@
         <v>0</v>
       </c>
       <c r="I248" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J248" t="s">
         <v>20</v>
       </c>
       <c r="K248" t="s">
+        <v>1302</v>
+      </c>
+      <c r="L248" t="s">
+        <v>19</v>
+      </c>
+      <c r="M248" t="s">
+        <v>22</v>
+      </c>
+      <c r="N248" t="s">
         <v>1303</v>
       </c>
-      <c r="L248" t="s">
-        <v>19</v>
-      </c>
-      <c r="M248" t="s">
-        <v>22</v>
-      </c>
-      <c r="N248" t="s">
+      <c r="O248" t="s">
         <v>1304</v>
       </c>
-      <c r="O248" t="s">
+      <c r="P248" t="s">
         <v>1305</v>
-      </c>
-      <c r="P248" t="s">
-        <v>1306</v>
       </c>
     </row>
     <row r="249" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="B249" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C249" t="s">
         <v>18</v>
@@ -16943,36 +16940,36 @@
         <v>0</v>
       </c>
       <c r="I249" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J249" t="s">
         <v>20</v>
       </c>
       <c r="K249" t="s">
+        <v>1307</v>
+      </c>
+      <c r="L249" t="s">
+        <v>19</v>
+      </c>
+      <c r="M249" t="s">
+        <v>22</v>
+      </c>
+      <c r="N249" t="s">
         <v>1308</v>
       </c>
-      <c r="L249" t="s">
-        <v>19</v>
-      </c>
-      <c r="M249" t="s">
-        <v>22</v>
-      </c>
-      <c r="N249" t="s">
+      <c r="O249" t="s">
         <v>1309</v>
       </c>
-      <c r="O249" t="s">
+      <c r="P249" t="s">
         <v>1310</v>
-      </c>
-      <c r="P249" t="s">
-        <v>1311</v>
       </c>
     </row>
     <row r="250" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="B250" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C250" t="s">
         <v>18</v>
@@ -16999,27 +16996,27 @@
         <v>20</v>
       </c>
       <c r="K250" t="s">
+        <v>1312</v>
+      </c>
+      <c r="L250" t="s">
+        <v>19</v>
+      </c>
+      <c r="M250" t="s">
+        <v>22</v>
+      </c>
+      <c r="N250" t="s">
         <v>1313</v>
       </c>
-      <c r="L250" t="s">
-        <v>19</v>
-      </c>
-      <c r="M250" t="s">
-        <v>22</v>
-      </c>
-      <c r="N250" t="s">
+      <c r="O250" t="s">
         <v>1314</v>
       </c>
-      <c r="O250" t="s">
+      <c r="P250" t="s">
         <v>1315</v>
-      </c>
-      <c r="P250" t="s">
-        <v>1316</v>
       </c>
     </row>
     <row r="251" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="B251" t="s">
         <v>19</v>
@@ -17049,7 +17046,7 @@
         <v>19</v>
       </c>
       <c r="K251" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="L251" t="s">
         <v>19</v>
@@ -17058,21 +17055,21 @@
         <v>326</v>
       </c>
       <c r="N251" t="s">
+        <v>1318</v>
+      </c>
+      <c r="O251" t="s">
+        <v>19</v>
+      </c>
+      <c r="P251" t="s">
         <v>1319</v>
-      </c>
-      <c r="O251" t="s">
-        <v>19</v>
-      </c>
-      <c r="P251" t="s">
-        <v>1320</v>
       </c>
     </row>
     <row r="252" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="B252" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C252" t="s">
         <v>18</v>
@@ -17093,36 +17090,36 @@
         <v>0</v>
       </c>
       <c r="I252" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J252" t="s">
         <v>20</v>
       </c>
       <c r="K252" t="s">
+        <v>1321</v>
+      </c>
+      <c r="L252" t="s">
+        <v>19</v>
+      </c>
+      <c r="M252" t="s">
+        <v>22</v>
+      </c>
+      <c r="N252" t="s">
         <v>1322</v>
       </c>
-      <c r="L252" t="s">
-        <v>19</v>
-      </c>
-      <c r="M252" t="s">
-        <v>22</v>
-      </c>
-      <c r="N252" t="s">
+      <c r="O252" t="s">
         <v>1323</v>
       </c>
-      <c r="O252" t="s">
-        <v>1324</v>
-      </c>
       <c r="P252" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="253" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="B253" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C253" t="s">
         <v>18</v>
@@ -17143,36 +17140,36 @@
         <v>0</v>
       </c>
       <c r="I253" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J253" t="s">
         <v>20</v>
       </c>
       <c r="K253" t="s">
+        <v>1325</v>
+      </c>
+      <c r="L253" t="s">
+        <v>19</v>
+      </c>
+      <c r="M253" t="s">
+        <v>22</v>
+      </c>
+      <c r="N253" t="s">
         <v>1326</v>
       </c>
-      <c r="L253" t="s">
-        <v>19</v>
-      </c>
-      <c r="M253" t="s">
-        <v>22</v>
-      </c>
-      <c r="N253" t="s">
+      <c r="O253" t="s">
         <v>1327</v>
       </c>
-      <c r="O253" t="s">
+      <c r="P253" t="s">
         <v>1328</v>
-      </c>
-      <c r="P253" t="s">
-        <v>1329</v>
       </c>
     </row>
     <row r="254" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="B254" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C254" t="s">
         <v>18</v>
@@ -17193,36 +17190,36 @@
         <v>0</v>
       </c>
       <c r="I254" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J254" t="s">
         <v>20</v>
       </c>
       <c r="K254" t="s">
+        <v>1330</v>
+      </c>
+      <c r="L254" t="s">
+        <v>19</v>
+      </c>
+      <c r="M254" t="s">
+        <v>22</v>
+      </c>
+      <c r="N254" t="s">
         <v>1331</v>
       </c>
-      <c r="L254" t="s">
-        <v>19</v>
-      </c>
-      <c r="M254" t="s">
-        <v>22</v>
-      </c>
-      <c r="N254" t="s">
+      <c r="O254" t="s">
         <v>1332</v>
       </c>
-      <c r="O254" t="s">
+      <c r="P254" t="s">
         <v>1333</v>
-      </c>
-      <c r="P254" t="s">
-        <v>1334</v>
       </c>
     </row>
     <row r="255" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B255" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C255" t="s">
         <v>18</v>
@@ -17243,36 +17240,36 @@
         <v>0</v>
       </c>
       <c r="I255" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J255" t="s">
         <v>20</v>
       </c>
       <c r="K255" t="s">
+        <v>1335</v>
+      </c>
+      <c r="L255" t="s">
+        <v>19</v>
+      </c>
+      <c r="M255" t="s">
+        <v>22</v>
+      </c>
+      <c r="N255" t="s">
         <v>1336</v>
       </c>
-      <c r="L255" t="s">
-        <v>19</v>
-      </c>
-      <c r="M255" t="s">
-        <v>22</v>
-      </c>
-      <c r="N255" t="s">
+      <c r="O255" t="s">
         <v>1337</v>
       </c>
-      <c r="O255" t="s">
+      <c r="P255" t="s">
         <v>1338</v>
-      </c>
-      <c r="P255" t="s">
-        <v>1339</v>
       </c>
     </row>
     <row r="256" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="B256" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C256" t="s">
         <v>18</v>
@@ -17293,36 +17290,36 @@
         <v>0</v>
       </c>
       <c r="I256" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J256" t="s">
         <v>20</v>
       </c>
       <c r="K256" t="s">
+        <v>1340</v>
+      </c>
+      <c r="L256" t="s">
+        <v>19</v>
+      </c>
+      <c r="M256" t="s">
+        <v>22</v>
+      </c>
+      <c r="N256" t="s">
         <v>1341</v>
       </c>
-      <c r="L256" t="s">
-        <v>19</v>
-      </c>
-      <c r="M256" t="s">
-        <v>22</v>
-      </c>
-      <c r="N256" t="s">
+      <c r="O256" t="s">
         <v>1342</v>
       </c>
-      <c r="O256" t="s">
+      <c r="P256" t="s">
         <v>1343</v>
-      </c>
-      <c r="P256" t="s">
-        <v>1344</v>
       </c>
     </row>
     <row r="257" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="B257" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C257" t="s">
         <v>18</v>
@@ -17343,33 +17340,33 @@
         <v>0</v>
       </c>
       <c r="I257" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J257" t="s">
         <v>20</v>
       </c>
       <c r="K257" t="s">
+        <v>1345</v>
+      </c>
+      <c r="L257" t="s">
+        <v>19</v>
+      </c>
+      <c r="M257" t="s">
+        <v>22</v>
+      </c>
+      <c r="N257" t="s">
         <v>1346</v>
       </c>
-      <c r="L257" t="s">
-        <v>19</v>
-      </c>
-      <c r="M257" t="s">
-        <v>22</v>
-      </c>
-      <c r="N257" t="s">
+      <c r="O257" t="s">
         <v>1347</v>
       </c>
-      <c r="O257" t="s">
+      <c r="P257" t="s">
         <v>1348</v>
-      </c>
-      <c r="P257" t="s">
-        <v>1349</v>
       </c>
     </row>
     <row r="258" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="B258" t="s">
         <v>18</v>
@@ -17399,7 +17396,7 @@
         <v>42</v>
       </c>
       <c r="K258" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="L258" t="b">
         <v>0</v>
@@ -17408,21 +17405,21 @@
         <v>22</v>
       </c>
       <c r="N258" t="s">
+        <v>1351</v>
+      </c>
+      <c r="O258" t="s">
         <v>1352</v>
       </c>
-      <c r="O258" t="s">
+      <c r="P258" t="s">
         <v>1353</v>
-      </c>
-      <c r="P258" t="s">
-        <v>1354</v>
       </c>
     </row>
     <row r="259" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="B259" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C259" t="s">
         <v>18</v>
@@ -17443,39 +17440,39 @@
         <v>0</v>
       </c>
       <c r="I259" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="J259" t="s">
         <v>20</v>
       </c>
       <c r="K259" t="s">
+        <v>1355</v>
+      </c>
+      <c r="L259" t="s">
+        <v>19</v>
+      </c>
+      <c r="M259" t="s">
+        <v>22</v>
+      </c>
+      <c r="N259" t="s">
         <v>1356</v>
       </c>
-      <c r="L259" t="s">
-        <v>19</v>
-      </c>
-      <c r="M259" t="s">
-        <v>22</v>
-      </c>
-      <c r="N259" t="s">
+      <c r="O259" t="s">
         <v>1357</v>
       </c>
-      <c r="O259" t="s">
+      <c r="P259" t="s">
         <v>1358</v>
-      </c>
-      <c r="P259" t="s">
-        <v>1359</v>
       </c>
     </row>
     <row r="260" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
+        <v>1359</v>
+      </c>
+      <c r="B260" t="s">
         <v>1360</v>
       </c>
-      <c r="B260" t="s">
+      <c r="C260" t="s">
         <v>1361</v>
-      </c>
-      <c r="C260" t="s">
-        <v>1362</v>
       </c>
       <c r="D260" t="b">
         <v>0</v>
@@ -17499,7 +17496,7 @@
         <v>42</v>
       </c>
       <c r="K260" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="L260" t="b">
         <v>1</v>
@@ -17508,13 +17505,13 @@
         <v>22</v>
       </c>
       <c r="N260" t="s">
+        <v>1363</v>
+      </c>
+      <c r="O260" t="s">
         <v>1364</v>
       </c>
-      <c r="O260" t="s">
+      <c r="P260" t="s">
         <v>1365</v>
-      </c>
-      <c r="P260" t="s">
-        <v>1366</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add columns, video blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (16):
- blocks/columns/columns.css
- blocks/video/overlay.js
- blocks/video/video.css
- styles/lazy-styles.css
- templates/contactus/contactus.css
- templates/sidebar/sidebar.css
- templates/sidebar/sidebar.js
- tools/importer/FORMS-INVENTORY.md
- tools/importer/LLM-ONBOARDING-PROMPT.md
- tools/importer/MIGRATION-PLAYBOOK.md
- tools/importer/PRODUCTS-QA-FINDINGS.md
- tools/importer/backups/products/MANIFEST.md
- tools/importer/reports/import-grace-master.report.xlsx
- tools/importer/reports/products/metallocenes.report.json
- tools/importer/reports/products/polytrak-catalysts.report.json
- tools/importer/reports/products/sylosiv.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-grace-master.report.xlsx
+++ b/tools/importer/reports/import-grace-master.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3664" uniqueCount="1366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3663" uniqueCount="1367">
   <si>
     <t>_reportFile</t>
   </si>
@@ -3153,7 +3153,10 @@
     <t>products/metallocenes</t>
   </si>
   <si>
-    <t>2026-08-11T20:16:13.549Z</t>
+    <t>2026-08-11T23:25:00.988Z</t>
+  </si>
+  <si>
+    <t>Metallocenes</t>
   </si>
   <si>
     <t>https://grace.com/products/metallocenes/</t>
@@ -3165,7 +3168,7 @@
     <t>products/polytrak-catalysts</t>
   </si>
   <si>
-    <t>2026-08-09T21:33:17.355Z</t>
+    <t>2026-08-11T23:25:53.875Z</t>
   </si>
   <si>
     <t>POLYTRAK® Catalysts</t>
@@ -3372,7 +3375,7 @@
     <t>products/sylosiv</t>
   </si>
   <si>
-    <t>2026-08-09T21:44:59.032Z</t>
+    <t>2026-08-11T23:26:48.052Z</t>
   </si>
   <si>
     <t>SYLOSIV®</t>
@@ -14519,10 +14522,10 @@
         <v>1044</v>
       </c>
       <c r="B201" t="s">
-        <v>19</v>
+        <v>979</v>
       </c>
       <c r="C201" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D201" t="s">
         <v>19</v>
@@ -14531,19 +14534,19 @@
         <v>19</v>
       </c>
       <c r="F201" t="s">
-        <v>323</v>
+        <v>19</v>
       </c>
       <c r="G201" t="s">
-        <v>324</v>
-      </c>
-      <c r="H201" t="s">
-        <v>19</v>
+        <v>19</v>
+      </c>
+      <c r="H201" t="b">
+        <v>0</v>
       </c>
       <c r="I201" t="s">
-        <v>19</v>
+        <v>980</v>
       </c>
       <c r="J201" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K201" t="s">
         <v>1045</v>
@@ -14552,21 +14555,21 @@
         <v>19</v>
       </c>
       <c r="M201" t="s">
-        <v>326</v>
+        <v>22</v>
       </c>
       <c r="N201" t="s">
         <v>1046</v>
       </c>
       <c r="O201" t="s">
-        <v>19</v>
+        <v>1047</v>
       </c>
       <c r="P201" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="202" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="B202" t="s">
         <v>979</v>
@@ -14596,7 +14599,7 @@
         <v>20</v>
       </c>
       <c r="K202" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="L202" t="s">
         <v>19</v>
@@ -14605,21 +14608,21 @@
         <v>22</v>
       </c>
       <c r="N202" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="O202" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="P202" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="203" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="B203" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="C203" t="s">
         <v>18</v>
@@ -14646,7 +14649,7 @@
         <v>42</v>
       </c>
       <c r="K203" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="L203" t="b">
         <v>1</v>
@@ -14655,18 +14658,18 @@
         <v>22</v>
       </c>
       <c r="N203" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="O203" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="P203" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="204" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="B204" t="s">
         <v>18</v>
@@ -14696,7 +14699,7 @@
         <v>42</v>
       </c>
       <c r="K204" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="L204" t="b">
         <v>1</v>
@@ -14705,21 +14708,21 @@
         <v>22</v>
       </c>
       <c r="N204" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="O204" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="P204" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="205" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="B205" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="C205" t="s">
         <v>18</v>
@@ -14746,7 +14749,7 @@
         <v>20</v>
       </c>
       <c r="K205" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="L205" t="s">
         <v>19</v>
@@ -14755,18 +14758,18 @@
         <v>22</v>
       </c>
       <c r="N205" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="O205" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="P205" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="206" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="B206" t="s">
         <v>979</v>
@@ -14796,7 +14799,7 @@
         <v>20</v>
       </c>
       <c r="K206" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="L206" t="s">
         <v>19</v>
@@ -14805,21 +14808,21 @@
         <v>22</v>
       </c>
       <c r="N206" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="O206" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="P206" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="207" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="B207" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="C207" t="s">
         <v>18</v>
@@ -14846,7 +14849,7 @@
         <v>20</v>
       </c>
       <c r="K207" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="L207" t="s">
         <v>19</v>
@@ -14855,18 +14858,18 @@
         <v>22</v>
       </c>
       <c r="N207" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="O207" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="P207" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="208" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="B208" t="s">
         <v>1024</v>
@@ -14896,7 +14899,7 @@
         <v>20</v>
       </c>
       <c r="K208" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="L208" t="s">
         <v>19</v>
@@ -14905,21 +14908,21 @@
         <v>22</v>
       </c>
       <c r="N208" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="O208" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="P208" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="209" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="B209" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="C209" t="s">
         <v>18</v>
@@ -14946,7 +14949,7 @@
         <v>20</v>
       </c>
       <c r="K209" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="L209" t="s">
         <v>19</v>
@@ -14955,21 +14958,21 @@
         <v>22</v>
       </c>
       <c r="N209" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="O209" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="P209" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="210" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="B210" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="C210" t="s">
         <v>18</v>
@@ -14996,7 +14999,7 @@
         <v>20</v>
       </c>
       <c r="K210" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="L210" t="s">
         <v>19</v>
@@ -15005,21 +15008,21 @@
         <v>22</v>
       </c>
       <c r="N210" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="O210" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="P210" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="211" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="B211" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="C211" t="s">
         <v>18</v>
@@ -15046,7 +15049,7 @@
         <v>20</v>
       </c>
       <c r="K211" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="L211" t="s">
         <v>19</v>
@@ -15055,21 +15058,21 @@
         <v>22</v>
       </c>
       <c r="N211" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="O211" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="P211" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="212" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="B212" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="C212" t="s">
         <v>18</v>
@@ -15096,7 +15099,7 @@
         <v>20</v>
       </c>
       <c r="K212" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="L212" t="s">
         <v>19</v>
@@ -15105,18 +15108,18 @@
         <v>22</v>
       </c>
       <c r="N212" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="O212" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="P212" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="213" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="B213" t="s">
         <v>979</v>
@@ -15146,7 +15149,7 @@
         <v>20</v>
       </c>
       <c r="K213" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="L213" t="s">
         <v>19</v>
@@ -15155,18 +15158,18 @@
         <v>22</v>
       </c>
       <c r="N213" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="O213" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="P213" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="214" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="B214" t="s">
         <v>979</v>
@@ -15196,7 +15199,7 @@
         <v>20</v>
       </c>
       <c r="K214" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="L214" t="s">
         <v>19</v>
@@ -15205,18 +15208,18 @@
         <v>22</v>
       </c>
       <c r="N214" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="O214" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="P214" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="215" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="B215" t="s">
         <v>1024</v>
@@ -15246,7 +15249,7 @@
         <v>20</v>
       </c>
       <c r="K215" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="L215" t="s">
         <v>19</v>
@@ -15255,18 +15258,18 @@
         <v>22</v>
       </c>
       <c r="N215" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="O215" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="P215" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="216" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="B216" t="s">
         <v>18</v>
@@ -15296,7 +15299,7 @@
         <v>42</v>
       </c>
       <c r="K216" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="L216" t="b">
         <v>1</v>
@@ -15305,21 +15308,21 @@
         <v>22</v>
       </c>
       <c r="N216" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="O216" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="P216" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="217" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B217" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="C217" t="s">
         <v>18</v>
@@ -15346,7 +15349,7 @@
         <v>20</v>
       </c>
       <c r="K217" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="L217" t="s">
         <v>19</v>
@@ -15355,21 +15358,21 @@
         <v>22</v>
       </c>
       <c r="N217" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="O217" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="P217" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="218" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="B218" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="C218" t="s">
         <v>18</v>
@@ -15396,7 +15399,7 @@
         <v>20</v>
       </c>
       <c r="K218" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="L218" t="s">
         <v>19</v>
@@ -15405,18 +15408,18 @@
         <v>22</v>
       </c>
       <c r="N218" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="O218" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="P218" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="219" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="B219" t="s">
         <v>979</v>
@@ -15446,7 +15449,7 @@
         <v>20</v>
       </c>
       <c r="K219" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="L219" t="s">
         <v>19</v>
@@ -15455,21 +15458,21 @@
         <v>22</v>
       </c>
       <c r="N219" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="O219" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="P219" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="220" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="B220" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="C220" t="s">
         <v>18</v>
@@ -15496,7 +15499,7 @@
         <v>20</v>
       </c>
       <c r="K220" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="L220" t="s">
         <v>19</v>
@@ -15505,18 +15508,18 @@
         <v>22</v>
       </c>
       <c r="N220" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="O220" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="P220" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="221" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="B221" t="s">
         <v>979</v>
@@ -15546,7 +15549,7 @@
         <v>20</v>
       </c>
       <c r="K221" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="L221" t="s">
         <v>19</v>
@@ -15555,21 +15558,21 @@
         <v>22</v>
       </c>
       <c r="N221" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="O221" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="P221" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="222" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="B222" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="C222" t="s">
         <v>18</v>
@@ -15596,7 +15599,7 @@
         <v>20</v>
       </c>
       <c r="K222" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="L222" t="s">
         <v>19</v>
@@ -15605,24 +15608,24 @@
         <v>22</v>
       </c>
       <c r="N222" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="O222" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="P222" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="223" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="B223" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="C223" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="D223" t="s">
         <v>19</v>
@@ -15646,7 +15649,7 @@
         <v>20</v>
       </c>
       <c r="K223" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="L223" t="s">
         <v>19</v>
@@ -15655,21 +15658,21 @@
         <v>22</v>
       </c>
       <c r="N223" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="O223" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="P223" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="224" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="B224" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="C224" t="s">
         <v>18</v>
@@ -15696,7 +15699,7 @@
         <v>42</v>
       </c>
       <c r="K224" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="L224" t="b">
         <v>0</v>
@@ -15705,21 +15708,21 @@
         <v>22</v>
       </c>
       <c r="N224" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="O224" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="P224" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="225" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="B225" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="C225" t="s">
         <v>129</v>
@@ -15746,7 +15749,7 @@
         <v>42</v>
       </c>
       <c r="K225" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="L225" t="b">
         <v>1</v>
@@ -15755,21 +15758,21 @@
         <v>22</v>
       </c>
       <c r="N225" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="O225" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="P225" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="226" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="B226" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="C226" t="s">
         <v>18</v>
@@ -15796,7 +15799,7 @@
         <v>42</v>
       </c>
       <c r="K226" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="L226" t="b">
         <v>1</v>
@@ -15805,21 +15808,21 @@
         <v>22</v>
       </c>
       <c r="N226" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="O226" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="P226" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="227" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="B227" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="C227" t="s">
         <v>18</v>
@@ -15846,7 +15849,7 @@
         <v>20</v>
       </c>
       <c r="K227" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="L227" t="s">
         <v>19</v>
@@ -15855,21 +15858,21 @@
         <v>22</v>
       </c>
       <c r="N227" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="O227" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="P227" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="228" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="B228" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="C228" t="s">
         <v>18</v>
@@ -15896,7 +15899,7 @@
         <v>20</v>
       </c>
       <c r="K228" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="L228" t="s">
         <v>19</v>
@@ -15905,21 +15908,21 @@
         <v>22</v>
       </c>
       <c r="N228" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="O228" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="P228" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="229" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="B229" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="C229" t="s">
         <v>40</v>
@@ -15946,7 +15949,7 @@
         <v>42</v>
       </c>
       <c r="K229" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="L229" t="b">
         <v>1</v>
@@ -15955,21 +15958,21 @@
         <v>22</v>
       </c>
       <c r="N229" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="O229" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="P229" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="230" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="B230" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="C230" t="s">
         <v>18</v>
@@ -15990,13 +15993,13 @@
         <v>0</v>
       </c>
       <c r="I230" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J230" t="s">
         <v>20</v>
       </c>
       <c r="K230" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="L230" t="s">
         <v>19</v>
@@ -16005,24 +16008,24 @@
         <v>22</v>
       </c>
       <c r="N230" t="s">
-        <v>1208</v>
+        <v>1209</v>
       </c>
       <c r="O230" t="s">
-        <v>1209</v>
+        <v>1210</v>
       </c>
       <c r="P230" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="231" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="B231" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="C231" t="s">
-        <v>1213</v>
+        <v>1214</v>
       </c>
       <c r="D231" t="b">
         <v>0</v>
@@ -16046,7 +16049,7 @@
         <v>42</v>
       </c>
       <c r="K231" t="s">
-        <v>1214</v>
+        <v>1215</v>
       </c>
       <c r="L231" t="b">
         <v>1</v>
@@ -16055,24 +16058,24 @@
         <v>22</v>
       </c>
       <c r="N231" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="O231" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="P231" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="232" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>1218</v>
+        <v>1219</v>
       </c>
       <c r="B232" t="s">
-        <v>1219</v>
+        <v>1220</v>
       </c>
       <c r="C232" t="s">
-        <v>1220</v>
+        <v>1221</v>
       </c>
       <c r="D232" t="b">
         <v>0</v>
@@ -16096,7 +16099,7 @@
         <v>42</v>
       </c>
       <c r="K232" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="L232" t="b">
         <v>1</v>
@@ -16105,21 +16108,21 @@
         <v>22</v>
       </c>
       <c r="N232" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="O232" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="P232" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="233" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="B233" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C233" t="s">
         <v>18</v>
@@ -16146,7 +16149,7 @@
         <v>20</v>
       </c>
       <c r="K233" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="L233" t="s">
         <v>19</v>
@@ -16155,21 +16158,21 @@
         <v>22</v>
       </c>
       <c r="N233" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="O233" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="P233" t="s">
-        <v>1230</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="234" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="B234" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C234" t="s">
         <v>18</v>
@@ -16196,7 +16199,7 @@
         <v>20</v>
       </c>
       <c r="K234" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
       <c r="L234" t="s">
         <v>19</v>
@@ -16205,21 +16208,21 @@
         <v>22</v>
       </c>
       <c r="N234" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="O234" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="P234" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="235" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="B235" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C235" t="s">
         <v>18</v>
@@ -16246,7 +16249,7 @@
         <v>20</v>
       </c>
       <c r="K235" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="L235" t="s">
         <v>19</v>
@@ -16255,21 +16258,21 @@
         <v>22</v>
       </c>
       <c r="N235" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="O235" t="s">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="P235" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="236" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="B236" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C236" t="s">
         <v>18</v>
@@ -16296,7 +16299,7 @@
         <v>20</v>
       </c>
       <c r="K236" t="s">
-        <v>1242</v>
+        <v>1243</v>
       </c>
       <c r="L236" t="s">
         <v>19</v>
@@ -16305,21 +16308,21 @@
         <v>22</v>
       </c>
       <c r="N236" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="O236" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="P236" t="s">
-        <v>1245</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="237" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="B237" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C237" t="s">
         <v>18</v>
@@ -16346,7 +16349,7 @@
         <v>20</v>
       </c>
       <c r="K237" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="L237" t="s">
         <v>19</v>
@@ -16355,21 +16358,21 @@
         <v>22</v>
       </c>
       <c r="N237" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="O237" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="P237" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="238" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="B238" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C238" t="s">
         <v>18</v>
@@ -16396,7 +16399,7 @@
         <v>20</v>
       </c>
       <c r="K238" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="L238" t="s">
         <v>19</v>
@@ -16405,21 +16408,21 @@
         <v>22</v>
       </c>
       <c r="N238" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="O238" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="P238" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="239" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="B239" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C239" t="s">
         <v>18</v>
@@ -16446,7 +16449,7 @@
         <v>20</v>
       </c>
       <c r="K239" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
       <c r="L239" t="s">
         <v>19</v>
@@ -16455,21 +16458,21 @@
         <v>22</v>
       </c>
       <c r="N239" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="O239" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="P239" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="240" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="B240" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C240" t="s">
         <v>18</v>
@@ -16496,7 +16499,7 @@
         <v>20</v>
       </c>
       <c r="K240" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="L240" t="s">
         <v>19</v>
@@ -16505,21 +16508,21 @@
         <v>22</v>
       </c>
       <c r="N240" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="O240" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="P240" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="241" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="B241" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C241" t="s">
         <v>18</v>
@@ -16546,7 +16549,7 @@
         <v>20</v>
       </c>
       <c r="K241" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="L241" t="s">
         <v>19</v>
@@ -16555,21 +16558,21 @@
         <v>22</v>
       </c>
       <c r="N241" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="O241" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="P241" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="242" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="B242" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C242" t="s">
         <v>18</v>
@@ -16596,7 +16599,7 @@
         <v>20</v>
       </c>
       <c r="K242" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="L242" t="s">
         <v>19</v>
@@ -16605,21 +16608,21 @@
         <v>22</v>
       </c>
       <c r="N242" t="s">
-        <v>1273</v>
+        <v>1274</v>
       </c>
       <c r="O242" t="s">
-        <v>1274</v>
+        <v>1275</v>
       </c>
       <c r="P242" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="243" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="B243" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C243" t="s">
         <v>18</v>
@@ -16646,7 +16649,7 @@
         <v>20</v>
       </c>
       <c r="K243" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="L243" t="s">
         <v>19</v>
@@ -16655,21 +16658,21 @@
         <v>22</v>
       </c>
       <c r="N243" t="s">
-        <v>1278</v>
+        <v>1279</v>
       </c>
       <c r="O243" t="s">
-        <v>1279</v>
+        <v>1280</v>
       </c>
       <c r="P243" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="244" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>1281</v>
+        <v>1282</v>
       </c>
       <c r="B244" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C244" t="s">
         <v>18</v>
@@ -16696,7 +16699,7 @@
         <v>20</v>
       </c>
       <c r="K244" t="s">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="L244" t="s">
         <v>19</v>
@@ -16705,21 +16708,21 @@
         <v>22</v>
       </c>
       <c r="N244" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
       <c r="O244" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="P244" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="245" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>1286</v>
+        <v>1287</v>
       </c>
       <c r="B245" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C245" t="s">
         <v>18</v>
@@ -16740,13 +16743,13 @@
         <v>0</v>
       </c>
       <c r="I245" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J245" t="s">
         <v>20</v>
       </c>
       <c r="K245" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="L245" t="s">
         <v>19</v>
@@ -16755,21 +16758,21 @@
         <v>22</v>
       </c>
       <c r="N245" t="s">
-        <v>1288</v>
+        <v>1289</v>
       </c>
       <c r="O245" t="s">
-        <v>1289</v>
+        <v>1290</v>
       </c>
       <c r="P245" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="246" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="B246" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C246" t="s">
         <v>18</v>
@@ -16790,13 +16793,13 @@
         <v>0</v>
       </c>
       <c r="I246" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J246" t="s">
         <v>20</v>
       </c>
       <c r="K246" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="L246" t="s">
         <v>19</v>
@@ -16805,21 +16808,21 @@
         <v>22</v>
       </c>
       <c r="N246" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="O246" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="P246" t="s">
-        <v>1295</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="247" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>1296</v>
+        <v>1297</v>
       </c>
       <c r="B247" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C247" t="s">
         <v>18</v>
@@ -16840,13 +16843,13 @@
         <v>0</v>
       </c>
       <c r="I247" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J247" t="s">
         <v>20</v>
       </c>
       <c r="K247" t="s">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="L247" t="s">
         <v>19</v>
@@ -16855,21 +16858,21 @@
         <v>22</v>
       </c>
       <c r="N247" t="s">
-        <v>1298</v>
+        <v>1299</v>
       </c>
       <c r="O247" t="s">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="P247" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="248" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="B248" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C248" t="s">
         <v>18</v>
@@ -16890,13 +16893,13 @@
         <v>0</v>
       </c>
       <c r="I248" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J248" t="s">
         <v>20</v>
       </c>
       <c r="K248" t="s">
-        <v>1302</v>
+        <v>1303</v>
       </c>
       <c r="L248" t="s">
         <v>19</v>
@@ -16905,21 +16908,21 @@
         <v>22</v>
       </c>
       <c r="N248" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="O248" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
       <c r="P248" t="s">
-        <v>1305</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="249" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="B249" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C249" t="s">
         <v>18</v>
@@ -16940,13 +16943,13 @@
         <v>0</v>
       </c>
       <c r="I249" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J249" t="s">
         <v>20</v>
       </c>
       <c r="K249" t="s">
-        <v>1307</v>
+        <v>1308</v>
       </c>
       <c r="L249" t="s">
         <v>19</v>
@@ -16955,21 +16958,21 @@
         <v>22</v>
       </c>
       <c r="N249" t="s">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="O249" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="P249" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="250" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="B250" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C250" t="s">
         <v>18</v>
@@ -16996,7 +16999,7 @@
         <v>20</v>
       </c>
       <c r="K250" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="L250" t="s">
         <v>19</v>
@@ -17005,18 +17008,18 @@
         <v>22</v>
       </c>
       <c r="N250" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="O250" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="P250" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="251" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="B251" t="s">
         <v>19</v>
@@ -17046,7 +17049,7 @@
         <v>19</v>
       </c>
       <c r="K251" t="s">
-        <v>1317</v>
+        <v>1318</v>
       </c>
       <c r="L251" t="s">
         <v>19</v>
@@ -17055,21 +17058,21 @@
         <v>326</v>
       </c>
       <c r="N251" t="s">
-        <v>1318</v>
+        <v>1319</v>
       </c>
       <c r="O251" t="s">
         <v>19</v>
       </c>
       <c r="P251" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="252" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="B252" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C252" t="s">
         <v>18</v>
@@ -17090,13 +17093,13 @@
         <v>0</v>
       </c>
       <c r="I252" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J252" t="s">
         <v>20</v>
       </c>
       <c r="K252" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="L252" t="s">
         <v>19</v>
@@ -17105,21 +17108,21 @@
         <v>22</v>
       </c>
       <c r="N252" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="O252" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="P252" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="253" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="B253" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C253" t="s">
         <v>18</v>
@@ -17140,13 +17143,13 @@
         <v>0</v>
       </c>
       <c r="I253" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J253" t="s">
         <v>20</v>
       </c>
       <c r="K253" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="L253" t="s">
         <v>19</v>
@@ -17155,21 +17158,21 @@
         <v>22</v>
       </c>
       <c r="N253" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="O253" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="P253" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="254" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="B254" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C254" t="s">
         <v>18</v>
@@ -17190,13 +17193,13 @@
         <v>0</v>
       </c>
       <c r="I254" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J254" t="s">
         <v>20</v>
       </c>
       <c r="K254" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="L254" t="s">
         <v>19</v>
@@ -17205,21 +17208,21 @@
         <v>22</v>
       </c>
       <c r="N254" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="O254" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="P254" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="255" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="B255" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C255" t="s">
         <v>18</v>
@@ -17240,13 +17243,13 @@
         <v>0</v>
       </c>
       <c r="I255" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J255" t="s">
         <v>20</v>
       </c>
       <c r="K255" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="L255" t="s">
         <v>19</v>
@@ -17255,21 +17258,21 @@
         <v>22</v>
       </c>
       <c r="N255" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="O255" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="P255" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="256" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="B256" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C256" t="s">
         <v>18</v>
@@ -17290,13 +17293,13 @@
         <v>0</v>
       </c>
       <c r="I256" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J256" t="s">
         <v>20</v>
       </c>
       <c r="K256" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="L256" t="s">
         <v>19</v>
@@ -17305,21 +17308,21 @@
         <v>22</v>
       </c>
       <c r="N256" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="O256" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="P256" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="257" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
       <c r="B257" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C257" t="s">
         <v>18</v>
@@ -17340,13 +17343,13 @@
         <v>0</v>
       </c>
       <c r="I257" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J257" t="s">
         <v>20</v>
       </c>
       <c r="K257" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="L257" t="s">
         <v>19</v>
@@ -17355,18 +17358,18 @@
         <v>22</v>
       </c>
       <c r="N257" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="O257" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="P257" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="258" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="B258" t="s">
         <v>18</v>
@@ -17396,7 +17399,7 @@
         <v>42</v>
       </c>
       <c r="K258" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
       <c r="L258" t="b">
         <v>0</v>
@@ -17405,21 +17408,21 @@
         <v>22</v>
       </c>
       <c r="N258" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
       <c r="O258" t="s">
-        <v>1352</v>
+        <v>1353</v>
       </c>
       <c r="P258" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="259" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="B259" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C259" t="s">
         <v>18</v>
@@ -17440,13 +17443,13 @@
         <v>0</v>
       </c>
       <c r="I259" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="J259" t="s">
         <v>20</v>
       </c>
       <c r="K259" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="L259" t="s">
         <v>19</v>
@@ -17455,24 +17458,24 @@
         <v>22</v>
       </c>
       <c r="N259" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="O259" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="P259" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="260" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="B260" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="C260" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="D260" t="b">
         <v>0</v>
@@ -17496,7 +17499,7 @@
         <v>42</v>
       </c>
       <c r="K260" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="L260" t="b">
         <v>1</v>
@@ -17505,13 +17508,13 @@
         <v>22</v>
       </c>
       <c r="N260" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="O260" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="P260" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
     </row>
   </sheetData>

</xml_diff>